<commit_message>
feat(excel-to-pdf): 新增 PdfHelper 流式 API，懒加载至终端操作才构建 PDF
- 新增 helper 包：PdfHelper 门面提供 classpath 模板、模板字节、已填充 Excel 四种静态入口
- 链按 PdfTemplateChain / PdfTerminal 接口类型收窄 API：excel 链编译期即无填充方法，删除运行时来源校验
- 三种终端操作 toByteArray / toFile / toBrowser 首次调用才懒构建（读模板 → ExcelUtil 生成 xlsx → LibreOffice 转
  PDF）并缓存，同链多次终端操作不重复转换
- 填充方法 appendSheet / appendSheets（追加）与 sheets（整体替换），List.copyOf 做快照并拒绝 null 元素
- LibreOffice 转换配置由 PdfHelperConfiguration 启动时注册为全局默认，链构造器快照，脱离 Spring 自动回退内置默认值
- 新增 PdfHelperManualCheckTest：一测试方法一情况，覆盖三种入口、三个终端操作、懒构建缓存复用与空 Sheet 规则断言
- PDFUtil 重命名为 PdfUtil，同步模块内引用与 architecture.md 描述
- README 增补 PdfHelper 流式 API 小节与测试产物说明
</commit_message>
<xml_diff>
--- a/excel-to-pdf/src/main/resources/excel-template/template.xlsx
+++ b/excel-to-pdf/src/main/resources/excel-template/template.xlsx
@@ -1309,15 +1309,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:J4"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="3"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="10" width="12" customWidth="1"/>
+    <col min="1" max="1" width="13.25" customWidth="1"/>
+    <col min="2" max="2" width="15.125" customWidth="1"/>
+    <col min="3" max="3" width="17.375" customWidth="1"/>
+    <col min="4" max="4" width="15.875" customWidth="1"/>
+    <col min="5" max="6" width="17.125" customWidth="1"/>
+    <col min="7" max="7" width="18.375" customWidth="1"/>
+    <col min="8" max="8" width="16.75" customWidth="1"/>
+    <col min="9" max="9" width="18.25" customWidth="1"/>
+    <col min="10" max="10" width="17.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" spans="1:10">
@@ -1366,7 +1372,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:10">
+    <row r="3" s="1" customFormat="1" ht="36" customHeight="1" spans="1:10">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -1398,7 +1404,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" ht="32" customHeight="1" spans="1:10">
       <c r="A4" s="6" t="s">
         <v>11</v>
       </c>
@@ -1417,7 +1423,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A4:J4"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.298611111111111" footer="0.298611111111111"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>